<commit_message>
Adicion de las imagenes de los mapas de huevos y larvas
</commit_message>
<xml_diff>
--- a/data/raw/maps/Coordenadas_Corregido_mapa_Icito_Sin2019.xlsx
+++ b/data/raw/maps/Coordenadas_Corregido_mapa_Icito_Sin2019.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\home\chrisbermudezr\IchthyoplanktonERFEN\data\raw\maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08286916-1829-436B-89CE-2ED6CB58A7A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75284E2A-7CD7-448A-B0F7-A64F672CEEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-70" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapas_Christian" sheetId="1" r:id="rId1"/>
@@ -7136,805 +7136,1687 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BEB52C1-D0E4-40CD-A712-43B440F55F9C}">
-  <dimension ref="A1:A191"/>
+  <dimension ref="A1:G191"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1">
         <v>11819.46</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D1">
+        <v>101809</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>8739.84</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D2">
+        <v>73541</v>
+      </c>
+      <c r="G2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>3905.37</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D3">
+        <v>62066</v>
+      </c>
+      <c r="G3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3731.34</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D4">
+        <v>61161</v>
+      </c>
+      <c r="G4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2947.32</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D5">
+        <v>59212</v>
+      </c>
+      <c r="G5">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2751.46</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <v>34236</v>
+      </c>
+      <c r="G6">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2610.7600000000002</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D7">
+        <v>26886</v>
+      </c>
+      <c r="G7">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2331.19</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D8">
+        <v>24756</v>
+      </c>
+      <c r="G8">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1931.11</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D9">
+        <v>22815</v>
+      </c>
+      <c r="G9">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1886.11</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D10">
+        <v>22035</v>
+      </c>
+      <c r="G10">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1869.98</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <v>18123</v>
+      </c>
+      <c r="G11">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1862.63</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D12">
+        <v>15314</v>
+      </c>
+      <c r="G12">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1803.42</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D13">
+        <v>13923</v>
+      </c>
+      <c r="G13">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1711.03</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D14">
+        <v>13029</v>
+      </c>
+      <c r="G14">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1683.89</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D15">
+        <v>11257</v>
+      </c>
+      <c r="G15">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1515.24</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D16">
+        <v>10696</v>
+      </c>
+      <c r="G16">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1356.7</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D17">
+        <v>10298</v>
+      </c>
+      <c r="G17">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1321.9</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D18">
+        <v>8973</v>
+      </c>
+      <c r="G18">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1091.23</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D19">
+        <v>8864</v>
+      </c>
+      <c r="G19">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1035.44</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D20">
+        <v>5885</v>
+      </c>
+      <c r="G20">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>863.11</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D21">
+        <v>5846</v>
+      </c>
+      <c r="G21">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>854.99</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D22">
+        <v>5702</v>
+      </c>
+      <c r="G22">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>833.82</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D23">
+        <v>5695</v>
+      </c>
+      <c r="G23">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>815.49</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D24">
+        <v>5187.42</v>
+      </c>
+      <c r="G24">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>753.37</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D25">
+        <v>5154</v>
+      </c>
+      <c r="G25">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>729.88</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D26">
+        <v>4893</v>
+      </c>
+      <c r="G26">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>722.41</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D27">
+        <v>4595</v>
+      </c>
+      <c r="G27">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>715.93</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D28">
+        <v>4371</v>
+      </c>
+      <c r="G28">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>669.55</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D29">
+        <v>4266</v>
+      </c>
+      <c r="G29">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>662.25</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D30">
+        <v>4020</v>
+      </c>
+      <c r="G30">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>643.87</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D31">
+        <v>3721</v>
+      </c>
+      <c r="G31">
+        <v>368.64</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>594.4</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D32">
+        <v>3388</v>
+      </c>
+      <c r="G32">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>585.55999999999995</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D33">
+        <v>3187</v>
+      </c>
+      <c r="G33">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>577.73</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D34">
+        <v>3135</v>
+      </c>
+      <c r="G34">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>548.79999999999995</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D35">
+        <v>2994</v>
+      </c>
+      <c r="G35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>537.80999999999995</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D36">
+        <v>2825</v>
+      </c>
+      <c r="G36">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>521.48</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D37">
+        <v>2793</v>
+      </c>
+      <c r="G37">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>506.55</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D38">
+        <v>2749</v>
+      </c>
+      <c r="G38">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>485.5</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D39">
+        <v>2504</v>
+      </c>
+      <c r="G39">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>455.62</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D40">
+        <v>2408</v>
+      </c>
+      <c r="G40">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>440.8</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D41">
+        <v>2278</v>
+      </c>
+      <c r="G41">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>429.25</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D42">
+        <v>2242</v>
+      </c>
+      <c r="G42">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>407.21</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D43">
+        <v>1913</v>
+      </c>
+      <c r="G43">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>385.21</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D44">
+        <v>1889</v>
+      </c>
+      <c r="G44">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>381.94</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D45">
+        <v>1820</v>
+      </c>
+      <c r="G45">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>363.92</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D46">
+        <v>1770</v>
+      </c>
+      <c r="G46">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>358.11</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D47">
+        <v>1766</v>
+      </c>
+      <c r="G47">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>355.63</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D48">
+        <v>1762</v>
+      </c>
+      <c r="G48">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>349.45</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D49">
+        <v>1662</v>
+      </c>
+      <c r="G49">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>346.38</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D50">
+        <v>1633</v>
+      </c>
+      <c r="G50">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>341.95</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D51">
+        <v>1630</v>
+      </c>
+      <c r="G51">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>341.94</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D52">
+        <v>1620</v>
+      </c>
+      <c r="G52">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>324.07</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D53">
+        <v>1532.16</v>
+      </c>
+      <c r="G53">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>322.47000000000003</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D54">
+        <v>1463</v>
+      </c>
+      <c r="G54">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>316.60000000000002</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D55">
+        <v>1458</v>
+      </c>
+      <c r="G55">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>302.11</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D56">
+        <v>1438</v>
+      </c>
+      <c r="G56">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>296.20999999999998</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D57">
+        <v>1328</v>
+      </c>
+      <c r="G57">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>289.93</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D58">
+        <v>1258</v>
+      </c>
+      <c r="G58">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>287.55</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D59">
+        <v>1166</v>
+      </c>
+      <c r="G59">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>267.24</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D60">
+        <v>1165</v>
+      </c>
+      <c r="G60">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>265.19</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D61">
+        <v>1137</v>
+      </c>
+      <c r="G61">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>262.76</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D62">
+        <v>1110</v>
+      </c>
+      <c r="G62">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>259.39999999999998</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D63">
+        <v>1065</v>
+      </c>
+      <c r="G63">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>251.83</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D64">
+        <v>1030</v>
+      </c>
+      <c r="G64">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>249.69</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D65">
+        <v>990</v>
+      </c>
+      <c r="G65">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>246.74</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D66">
+        <v>984</v>
+      </c>
+      <c r="G66">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>246.59</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D67">
+        <v>981</v>
+      </c>
+      <c r="G67">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>246.59</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D68">
+        <v>951</v>
+      </c>
+      <c r="G68">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>244.59</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D69">
+        <v>950</v>
+      </c>
+      <c r="G69">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>241.16</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D70">
+        <v>931</v>
+      </c>
+      <c r="G70">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>232.02</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D71">
+        <v>909</v>
+      </c>
+      <c r="G71">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>216.78</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D72">
+        <v>894</v>
+      </c>
+      <c r="G72">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>210</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D73">
+        <v>885</v>
+      </c>
+      <c r="G73">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>204.44</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D74">
+        <v>880</v>
+      </c>
+      <c r="G74">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>201.31</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D75">
+        <v>880</v>
+      </c>
+      <c r="G75">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>201.18</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D76">
+        <v>878</v>
+      </c>
+      <c r="G76">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>198.91</v>
       </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D77">
+        <v>829</v>
+      </c>
+      <c r="G77">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>196.1</v>
       </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D78">
+        <v>816</v>
+      </c>
+      <c r="G78">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>195.24</v>
       </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D79">
+        <v>789</v>
+      </c>
+      <c r="G79">
+        <v>720.2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>190.12</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D80">
+        <v>748</v>
+      </c>
+      <c r="G80">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>188.74</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D81">
+        <v>741</v>
+      </c>
+      <c r="G81">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>186.77</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D82">
+        <v>690</v>
+      </c>
+      <c r="G82">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>183.51</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D83">
+        <v>673</v>
+      </c>
+      <c r="G83">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>180.67</v>
       </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D84">
+        <v>663</v>
+      </c>
+      <c r="G84">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>179.87</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D85">
+        <v>658</v>
+      </c>
+      <c r="G85">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>178.86</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D86">
+        <v>647</v>
+      </c>
+      <c r="G86">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>178.4</v>
       </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D87">
+        <v>629</v>
+      </c>
+      <c r="G87">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>175.26</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D88">
+        <v>625</v>
+      </c>
+      <c r="G88">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>171.9</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D89">
+        <v>624</v>
+      </c>
+      <c r="G89">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>171.22</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D90">
+        <v>602</v>
+      </c>
+      <c r="G90">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>170.1</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D91">
+        <v>601</v>
+      </c>
+      <c r="G91">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>167.18</v>
       </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D92">
+        <v>593</v>
+      </c>
+      <c r="G92">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>163.1</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D93">
+        <v>576</v>
+      </c>
+      <c r="G93">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>158.9</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D94">
+        <v>569</v>
+      </c>
+      <c r="G94">
+        <v>932.1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>153.77000000000001</v>
       </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D95">
+        <v>565</v>
+      </c>
+      <c r="G95">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>147.88</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D96">
+        <v>550</v>
+      </c>
+      <c r="G96">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>147.76</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D97">
+        <v>540</v>
+      </c>
+      <c r="G97">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>146.19999999999999</v>
       </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D98">
+        <v>537</v>
+      </c>
+      <c r="G98">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>143.87</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D99">
+        <v>527</v>
+      </c>
+      <c r="G99">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>142.25</v>
       </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D100">
+        <v>523</v>
+      </c>
+      <c r="G100">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>141.75</v>
       </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D101">
+        <v>519</v>
+      </c>
+      <c r="G101">
+        <v>1019.94</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>141.46</v>
       </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D102">
+        <v>508</v>
+      </c>
+      <c r="G102">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>138.74</v>
       </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D103">
+        <v>506</v>
+      </c>
+      <c r="G103">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>135.99</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D104">
+        <v>441</v>
+      </c>
+      <c r="G104">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>135.03</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D105">
+        <v>428</v>
+      </c>
+      <c r="G105">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>134.97999999999999</v>
       </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D106">
+        <v>421</v>
+      </c>
+      <c r="G106">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>132.53</v>
       </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D107">
+        <v>404</v>
+      </c>
+      <c r="G107">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>127.41</v>
       </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D108">
+        <v>400</v>
+      </c>
+      <c r="G108">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>124.83</v>
       </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D109">
+        <v>383</v>
+      </c>
+      <c r="G109">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>123.04</v>
       </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D110">
+        <v>347</v>
+      </c>
+      <c r="G110">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>122.2</v>
       </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D111">
+        <v>342</v>
+      </c>
+      <c r="G111">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>121.9</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D112">
+        <v>329</v>
+      </c>
+      <c r="G112">
+        <v>1238</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>120.85</v>
       </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D113">
+        <v>327</v>
+      </c>
+      <c r="G113">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>118.9</v>
       </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D114">
+        <v>314</v>
+      </c>
+      <c r="G114">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>118.44</v>
       </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D115">
+        <v>308</v>
+      </c>
+      <c r="G115">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>117.84</v>
       </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D116">
+        <v>296</v>
+      </c>
+      <c r="G116">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116.97</v>
       </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D117">
+        <v>286</v>
+      </c>
+      <c r="G117">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>116.93</v>
       </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D118">
+        <v>282</v>
+      </c>
+      <c r="G118">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>115.68</v>
       </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D119">
+        <v>271</v>
+      </c>
+      <c r="G119">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>114.51</v>
       </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D120">
+        <v>265</v>
+      </c>
+      <c r="G120">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>113.07</v>
       </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D121">
+        <v>262</v>
+      </c>
+      <c r="G121">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>112.77</v>
       </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D122">
+        <v>249</v>
+      </c>
+      <c r="G122">
+        <v>1522.95</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>109.27</v>
       </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D123">
+        <v>233</v>
+      </c>
+      <c r="G123">
+        <v>1571</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>108.99</v>
       </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D124">
+        <v>233</v>
+      </c>
+      <c r="G124">
+        <v>1622.88</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>106.21</v>
       </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D125">
+        <v>233</v>
+      </c>
+      <c r="G125">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>105.5</v>
       </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D126">
+        <v>212</v>
+      </c>
+      <c r="G126">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>101.37</v>
       </c>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D127">
+        <v>200</v>
+      </c>
+      <c r="G127">
+        <v>1917</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>99.91</v>
       </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D128">
+        <v>198</v>
+      </c>
+      <c r="G128">
+        <v>1923</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>97.98</v>
       </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D129">
+        <v>176</v>
+      </c>
+      <c r="G129">
+        <v>1965</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>97.77</v>
       </c>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D130">
+        <v>166</v>
+      </c>
+      <c r="G130">
+        <v>1978</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>97.63</v>
       </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D131">
+        <v>137</v>
+      </c>
+      <c r="G131">
+        <v>2086</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>96.55</v>
       </c>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D132">
+        <v>137</v>
+      </c>
+      <c r="G132">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>95.42</v>
       </c>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D133">
+        <v>134</v>
+      </c>
+      <c r="G133">
+        <v>2319</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>89.21</v>
       </c>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D134">
+        <v>122</v>
+      </c>
+      <c r="G134">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>87.52</v>
       </c>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D135">
+        <v>71</v>
+      </c>
+      <c r="G135">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>86.97</v>
       </c>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D136">
+        <v>64</v>
+      </c>
+      <c r="G136">
+        <v>2446</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>86.31</v>
       </c>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D137">
+        <v>59</v>
+      </c>
+      <c r="G137">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>85.7</v>
       </c>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D138">
+        <v>59</v>
+      </c>
+      <c r="G138">
+        <v>2635</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>85.67</v>
       </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D139">
+        <v>55</v>
+      </c>
+      <c r="G139">
+        <v>2695</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>85.18</v>
       </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D140">
+        <v>40</v>
+      </c>
+      <c r="G140">
+        <v>2968</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>84.61</v>
       </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D141">
+        <v>32</v>
+      </c>
+      <c r="G141">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>84.19</v>
       </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D142">
+        <v>32</v>
+      </c>
+      <c r="G142">
+        <v>3601</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>83.3</v>
       </c>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D143">
+        <v>27</v>
+      </c>
+      <c r="G143">
+        <v>4039</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>83.02</v>
       </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D144">
+        <v>8</v>
+      </c>
+      <c r="G144">
+        <v>4243</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>81.3</v>
       </c>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="G145">
+        <v>4610</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>79.44</v>
       </c>
-    </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D146">
+        <v>0</v>
+      </c>
+      <c r="G146">
+        <v>5744</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>78.88</v>
       </c>
-    </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="D147">
+        <v>0</v>
+      </c>
+      <c r="G147">
+        <v>7657</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>77.849999999999994</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>76.84</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>76.67</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>70.95</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>68.44</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>65.66</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>64.42</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>63.27</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>63.22</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>62.56</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>61.59</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>61.31</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>60</v>
       </c>
@@ -8095,8 +8977,8 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A191">
-    <sortCondition descending="1" ref="A1:A191"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G1:G147">
+    <sortCondition ref="G1:G147"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>